<commit_message>
feat: estruturar planilha e adicionar relatorio de testes em HTML
</commit_message>
<xml_diff>
--- a/examples/report.xlsx
+++ b/examples/report.xlsx
@@ -8,8 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Dependências" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dependências'!$A$1:$J$7</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,14 +30,31 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="009C0006"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+        <bgColor rgb="001F3864"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -55,10 +75,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,313 +464,484 @@
   <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="33" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Versão requisitada</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Última versão PyPI</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Licença</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Última publicação</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Score Snyk</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Vulnerabilidades (total)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Vulnerabilidades (versão atual)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>flask</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>==3.1.3</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>3.1.3</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>A simple framework for building complex web applications.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>BSD-3-Clause</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>requests</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=2.31.0</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2.34.2</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Python HTTP for Humans.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>selenium</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=4.17.0</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>4.46.0</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Official Python bindings for Selenium WebDriver</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Apache-2.0</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>openpyxl</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=3.1.2</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>3.1.5</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>A Python library to read/write Excel 2010 xlsx/xlsm files</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>2024-06-28</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>pycrypto</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>==2.6.1</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>2.6.1</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Cryptographic modules for Python.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Public domain</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>2014-06-20</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>django</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>&gt;=4.2</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>6.0.7</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>A high-level Python web framework that encourages rapid development and clean, pragmatic design.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>BSD-3-Clause</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>158</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Coluna</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Significado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Nome da dependência conforme declarado no arquivo de entrada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Versão requisitada</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Especificador declarado no projeto, como "&gt;=3.0" ou "==2.6.1".</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Última versão PyPI</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Versão mais recente publicada no PyPI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Resumo do pacote informado pelo PyPI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Licença</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Licença declarada no PyPI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Última publicação</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Data da publicação mais recente no PyPI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Score Snyk</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Package Health Score do portal Snyk, de 0 a 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Vulnerabilidades (total)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Todas as vulnerabilidades já registradas para o pacote.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Vulnerabilidades (versão atual)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Quantas dessas ainda afetam a versão mais recente. É um subconjunto do total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>flask</t>
-        </is>
-      </c>
-      <c r="B2">
-        <f>=3.1.3</f>
-        <v/>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>3.1.3</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>A simple framework for building complex web applications.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>BSD-3-Clause</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>90</v>
-      </c>
-      <c r="H2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>requests</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>&gt;=2.31.0</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2.34.2</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Python HTTP for Humans.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Apache-2.0</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-05-14</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>91</v>
-      </c>
-      <c r="H3" t="n">
-        <v>10</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>selenium</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>&gt;=4.17.0</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>4.46.0</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Official Python bindings for Selenium WebDriver</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Apache-2.0</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-07-11</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>97</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>openpyxl</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>&gt;=3.1.2</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>3.1.5</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>A Python library to read/write Excel 2010 xlsx/xlsm files</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>MIT</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2024-06-28</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>pycrypto</t>
-        </is>
-      </c>
-      <c r="B6" s="2">
-        <f>=2.6.1</f>
-        <v/>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>2.6.1</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Cryptographic modules for Python.</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Public domain</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>2014-06-20</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>django</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>&gt;=4.2</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>6.0.7</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>A high-level Python web framework that encourages rapid development and clean, pragmatic design.</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>BSD-3-Clause</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>85</v>
-      </c>
-      <c r="H7" t="n">
-        <v>161</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Motivo de eventual falha na coleta dos dados da dependência.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Destaque em vermelho</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Dependências com Score Snyk inferior a 65. Pacotes sem score não são destacados: o dado está ausente, o que não significa nota ruim.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: cruzar vulnerabilidades do PyPI com as do Snyk
</commit_message>
<xml_diff>
--- a/examples/report.xlsx
+++ b/examples/report.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dependências'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dependências'!$A$1:$K$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -473,7 +473,8 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -524,6 +525,11 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Vulnerabilidades (PyPI/OSV)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Notas</t>
         </is>
       </c>
@@ -568,7 +574,10 @@
       <c r="I2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="2" t="n"/>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -610,7 +619,10 @@
       <c r="I3" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="2" t="n"/>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -652,7 +664,10 @@
       <c r="I4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="2" t="n"/>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -694,7 +709,10 @@
       <c r="I5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="2" t="n"/>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -736,7 +754,10 @@
       <c r="I6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="J6" s="4" t="n"/>
+      <c r="J6" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -770,18 +791,21 @@
         </is>
       </c>
       <c r="G7" s="3" t="n">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="2" t="n"/>
+      <c r="J7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:K7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -792,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -922,22 +946,34 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
+          <t>Vulnerabilidades (PyPI/OSV)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Vulnerabilidades na versão atual segundo a base OSV, informada pela API do PyPI. É uma fonte independente do Snyk: divergência entre as duas colunas significa que as bases avaliam de forma diferente quais versões são afetadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>Notas</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Motivo de eventual falha na coleta dos dados da dependência.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Destaque em vermelho</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Dependências com Score Snyk inferior a 65. Pacotes sem score não são destacados: o dado está ausente, o que não significa nota ruim.</t>
         </is>

</xml_diff>

<commit_message>
feat: adicionar aba de resumo estatistico
</commit_message>
<xml_diff>
--- a/examples/report.xlsx
+++ b/examples/report.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Dependências" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Legenda" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dependências'!$A$1:$K$7</definedName>
@@ -92,10 +93,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -816,7 +817,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Métrica</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dependências analisadas</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Com score abaixo de 65</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sem score no portal Snyk</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Pacotes com vulnerabilidade na versão atual</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Vulnerabilidades na versão atual (soma)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Vulnerabilidades no histórico (soma)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Divergências entre Snyk e OSV</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Falhas na coleta</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -824,19 +935,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Coluna</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Significado</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
@@ -848,7 +959,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Versão requisitada</t>
         </is>
@@ -860,7 +971,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Última versão PyPI</t>
         </is>
@@ -872,7 +983,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
@@ -884,7 +995,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Licença</t>
         </is>
@@ -896,7 +1007,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Última publicação</t>
         </is>
@@ -908,7 +1019,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Score Snyk</t>
         </is>
@@ -920,7 +1031,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Vulnerabilidades (total)</t>
         </is>
@@ -932,7 +1043,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Vulnerabilidades (versão atual)</t>
         </is>
@@ -944,7 +1055,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Vulnerabilidades (PyPI/OSV)</t>
         </is>
@@ -956,7 +1067,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -967,13 +1078,25 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Aba Resumo</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Visão geral da execução: totais, pacotes em risco e falhas de coleta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Destaque em vermelho</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Dependências com Score Snyk inferior a 65. Pacotes sem score não são destacados: o dado está ausente, o que não significa nota ruim.</t>
         </is>

</xml_diff>